<commit_message>
fix(config): prefer Azure API key for judge client; results/plot updates
_get_azure_client now auto-selects the API-key auth path when AZURE_OPENAI_API_KEY is set, falling back to az-login only when the key is absent. The DCA LLM judge (and midas eval) now work on machines without Azure CLI.

Also bundles in-progress results/plots + dca_experiments updates, tournament tweaks, and helper scripts (avg_tokens_old_repo.py, results/agentic).
</commit_message>
<xml_diff>
--- a/results/dca_experiments.xlsx
+++ b/results/dca_experiments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bosch-my.sharepoint.com/personal/bhs1rng_bosch_com/Documents/AIQ-212/Code/meta-prompting -16-07/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD912CC8-C306-4D1C-92EF-B06E15ADDFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{BD912CC8-C306-4D1C-92EF-B06E15ADDFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C34708CD-4893-4B53-9532-D9791B736318}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CA79904-42EF-4291-86DC-38C7E0E78A43}"/>
   </bookViews>
@@ -2322,25 +2322,22 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2356,21 +2353,24 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5156,16 +5156,16 @@
       </c>
     </row>
     <row r="29" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="121" t="s">
+      <c r="A29" s="120" t="s">
         <v>86</v>
       </c>
       <c r="B29" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="126" t="s">
+      <c r="C29" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="126"/>
+      <c r="D29" s="124"/>
       <c r="E29" s="6" t="s">
         <v>89</v>
       </c>
@@ -5197,7 +5197,7 @@
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A30" s="121"/>
+      <c r="A30" s="120"/>
       <c r="B30" s="21" t="s">
         <v>87</v>
       </c>
@@ -5238,7 +5238,7 @@
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A31" s="121"/>
+      <c r="A31" s="120"/>
       <c r="B31" s="21" t="s">
         <v>87</v>
       </c>
@@ -5277,14 +5277,14 @@
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A32" s="121"/>
+      <c r="A32" s="120"/>
       <c r="B32" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C32" s="131" t="s">
+      <c r="C32" s="125" t="s">
         <v>97</v>
       </c>
-      <c r="D32" s="131"/>
+      <c r="D32" s="125"/>
       <c r="E32" s="6" t="s">
         <v>98</v>
       </c>
@@ -5316,16 +5316,16 @@
       </c>
     </row>
     <row r="33" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="121" t="s">
+      <c r="A33" s="120" t="s">
         <v>101</v>
       </c>
-      <c r="B33" s="134" t="s">
+      <c r="B33" s="121" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="126" t="s">
+      <c r="C33" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D33" s="126"/>
+      <c r="D33" s="124"/>
       <c r="E33" s="6" t="s">
         <v>102</v>
       </c>
@@ -5362,8 +5362,8 @@
       </c>
     </row>
     <row r="34" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="121"/>
-      <c r="B34" s="135"/>
+      <c r="A34" s="120"/>
+      <c r="B34" s="122"/>
       <c r="C34" s="5" t="s">
         <v>88</v>
       </c>
@@ -5401,8 +5401,8 @@
       <c r="P34" s="6"/>
     </row>
     <row r="35" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="121"/>
-      <c r="B35" s="135"/>
+      <c r="A35" s="120"/>
+      <c r="B35" s="122"/>
       <c r="C35" s="5" t="s">
         <v>88</v>
       </c>
@@ -5440,8 +5440,8 @@
       <c r="P35" s="6"/>
     </row>
     <row r="36" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="121"/>
-      <c r="B36" s="135"/>
+      <c r="A36" s="120"/>
+      <c r="B36" s="122"/>
       <c r="C36" s="5" t="s">
         <v>88</v>
       </c>
@@ -5479,8 +5479,8 @@
       </c>
     </row>
     <row r="37" spans="1:17" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="121"/>
-      <c r="B37" s="135"/>
+      <c r="A37" s="120"/>
+      <c r="B37" s="122"/>
       <c r="C37" s="5" t="s">
         <v>88</v>
       </c>
@@ -5518,8 +5518,8 @@
       </c>
     </row>
     <row r="38" spans="1:17" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="121"/>
-      <c r="B38" s="136"/>
+      <c r="A38" s="120"/>
+      <c r="B38" s="123"/>
       <c r="C38" s="5" t="s">
         <v>88</v>
       </c>
@@ -5554,14 +5554,14 @@
       <c r="P38" s="6"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A39" s="121"/>
+      <c r="A39" s="120"/>
       <c r="B39" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C39" s="131" t="s">
+      <c r="C39" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="D39" s="131"/>
+      <c r="D39" s="125"/>
       <c r="E39" s="6" t="s">
         <v>141</v>
       </c>
@@ -5593,14 +5593,14 @@
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A40" s="121"/>
+      <c r="A40" s="120"/>
       <c r="B40" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C40" s="131" t="s">
+      <c r="C40" s="125" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="131"/>
+      <c r="D40" s="125"/>
       <c r="E40" s="6" t="s">
         <v>144</v>
       </c>
@@ -5632,14 +5632,14 @@
       </c>
     </row>
     <row r="41" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="121"/>
-      <c r="B41" s="127" t="s">
+      <c r="A41" s="120"/>
+      <c r="B41" s="126" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="126" t="s">
+      <c r="C41" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D41" s="126"/>
+      <c r="D41" s="124"/>
       <c r="E41" s="6" t="s">
         <v>148</v>
       </c>
@@ -5674,8 +5674,8 @@
       </c>
     </row>
     <row r="42" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="121"/>
-      <c r="B42" s="127"/>
+      <c r="A42" s="120"/>
+      <c r="B42" s="126"/>
       <c r="C42" s="5" t="s">
         <v>88</v>
       </c>
@@ -5716,8 +5716,8 @@
       </c>
     </row>
     <row r="43" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="121"/>
-      <c r="B43" s="127"/>
+      <c r="A43" s="120"/>
+      <c r="B43" s="126"/>
       <c r="C43" s="5" t="s">
         <v>88</v>
       </c>
@@ -5755,12 +5755,12 @@
       <c r="P43" s="6"/>
     </row>
     <row r="44" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="121"/>
-      <c r="B44" s="127"/>
-      <c r="C44" s="126" t="s">
+      <c r="A44" s="120"/>
+      <c r="B44" s="126"/>
+      <c r="C44" s="124" t="s">
         <v>166</v>
       </c>
-      <c r="D44" s="126"/>
+      <c r="D44" s="124"/>
       <c r="E44" s="6" t="s">
         <v>167</v>
       </c>
@@ -5792,8 +5792,8 @@
       <c r="P44" s="6"/>
     </row>
     <row r="45" spans="1:17" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="121"/>
-      <c r="B45" s="127"/>
+      <c r="A45" s="120"/>
+      <c r="B45" s="126"/>
       <c r="C45" s="5" t="s">
         <v>166</v>
       </c>
@@ -5831,8 +5831,8 @@
       </c>
     </row>
     <row r="46" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="121"/>
-      <c r="B46" s="127"/>
+      <c r="A46" s="120"/>
+      <c r="B46" s="126"/>
       <c r="C46" s="5" t="s">
         <v>166</v>
       </c>
@@ -5867,8 +5867,8 @@
       <c r="P46" s="6"/>
     </row>
     <row r="47" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="121"/>
-      <c r="B47" s="127"/>
+      <c r="A47" s="120"/>
+      <c r="B47" s="126"/>
       <c r="C47" s="5" t="s">
         <v>166</v>
       </c>
@@ -5903,14 +5903,14 @@
       <c r="P47" s="6"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A48" s="121"/>
+      <c r="A48" s="120"/>
       <c r="B48" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C48" s="131" t="s">
+      <c r="C48" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="D48" s="131"/>
+      <c r="D48" s="125"/>
       <c r="E48" s="6" t="s">
         <v>189</v>
       </c>
@@ -5940,14 +5940,14 @@
       <c r="P48" s="6"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A49" s="121"/>
+      <c r="A49" s="120"/>
       <c r="B49" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C49" s="131" t="s">
+      <c r="C49" s="125" t="s">
         <v>191</v>
       </c>
-      <c r="D49" s="131"/>
+      <c r="D49" s="125"/>
       <c r="E49" s="6" t="s">
         <v>192</v>
       </c>
@@ -5983,11 +5983,11 @@
       <c r="B50" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="126" t="s">
+      <c r="C50" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D50" s="126"/>
-      <c r="E50" s="123" t="s">
+      <c r="D50" s="124"/>
+      <c r="E50" s="133" t="s">
         <v>195</v>
       </c>
       <c r="F50" s="22">
@@ -6027,7 +6027,7 @@
       <c r="D51" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E51" s="124"/>
+      <c r="E51" s="134"/>
       <c r="F51" s="22">
         <v>0.70699999999999996</v>
       </c>
@@ -6059,11 +6059,11 @@
       <c r="B52" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C52" s="126" t="s">
+      <c r="C52" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D52" s="126"/>
-      <c r="E52" s="124"/>
+      <c r="D52" s="124"/>
+      <c r="E52" s="134"/>
       <c r="F52" s="22">
         <v>0.92700000000000005</v>
       </c>
@@ -6101,7 +6101,7 @@
       <c r="D53" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E53" s="124"/>
+      <c r="E53" s="134"/>
       <c r="F53" s="22">
         <v>0.878</v>
       </c>
@@ -6133,11 +6133,11 @@
       <c r="B54" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C54" s="126" t="s">
+      <c r="C54" s="124" t="s">
         <v>205</v>
       </c>
-      <c r="D54" s="126"/>
-      <c r="E54" s="124"/>
+      <c r="D54" s="124"/>
+      <c r="E54" s="134"/>
       <c r="F54" s="72" t="s">
         <v>206</v>
       </c>
@@ -6169,11 +6169,11 @@
       <c r="B55" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C55" s="126" t="s">
+      <c r="C55" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D55" s="126"/>
-      <c r="E55" s="124"/>
+      <c r="D55" s="124"/>
+      <c r="E55" s="134"/>
       <c r="F55" s="22">
         <v>0.93899999999999995</v>
       </c>
@@ -6211,7 +6211,7 @@
       <c r="D56" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E56" s="124"/>
+      <c r="E56" s="134"/>
       <c r="F56" s="22">
         <v>0.92700000000000005</v>
       </c>
@@ -6243,11 +6243,11 @@
       <c r="B57" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C57" s="126" t="s">
+      <c r="C57" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D57" s="126"/>
-      <c r="E57" s="124"/>
+      <c r="D57" s="124"/>
+      <c r="E57" s="134"/>
       <c r="F57" s="22">
         <v>0.92700000000000005</v>
       </c>
@@ -6285,7 +6285,7 @@
       <c r="D58" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E58" s="125"/>
+      <c r="E58" s="135"/>
       <c r="F58" s="22">
         <v>0.878</v>
       </c>
@@ -6317,11 +6317,11 @@
       <c r="B59" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C59" s="126" t="s">
+      <c r="C59" s="124" t="s">
         <v>205</v>
       </c>
-      <c r="D59" s="126"/>
-      <c r="E59" s="123" t="s">
+      <c r="D59" s="124"/>
+      <c r="E59" s="133" t="s">
         <v>219</v>
       </c>
       <c r="F59" s="22" t="s">
@@ -6355,11 +6355,11 @@
       <c r="B60" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C60" s="126" t="s">
+      <c r="C60" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="126"/>
-      <c r="E60" s="124"/>
+      <c r="D60" s="124"/>
+      <c r="E60" s="134"/>
       <c r="F60" s="22">
         <v>0.86599999999999999</v>
       </c>
@@ -6397,7 +6397,7 @@
       <c r="D61" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E61" s="124"/>
+      <c r="E61" s="134"/>
       <c r="F61" s="22">
         <v>0.78</v>
       </c>
@@ -6429,11 +6429,11 @@
       <c r="B62" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C62" s="126" t="s">
+      <c r="C62" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D62" s="126"/>
-      <c r="E62" s="124"/>
+      <c r="D62" s="124"/>
+      <c r="E62" s="134"/>
       <c r="F62" s="22">
         <v>0.82899999999999996</v>
       </c>
@@ -6471,7 +6471,7 @@
       <c r="D63" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E63" s="124"/>
+      <c r="E63" s="134"/>
       <c r="F63" s="22">
         <v>0.67100000000000004</v>
       </c>
@@ -6503,11 +6503,11 @@
       <c r="B64" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C64" s="126" t="s">
+      <c r="C64" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D64" s="126"/>
-      <c r="E64" s="124"/>
+      <c r="D64" s="124"/>
+      <c r="E64" s="134"/>
       <c r="F64" s="22">
         <v>0.81699999999999995</v>
       </c>
@@ -6545,7 +6545,7 @@
       <c r="D65" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E65" s="124"/>
+      <c r="E65" s="134"/>
       <c r="F65" s="22">
         <v>0.878</v>
       </c>
@@ -6577,11 +6577,11 @@
       <c r="B66" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C66" s="126" t="s">
+      <c r="C66" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D66" s="126"/>
-      <c r="E66" s="124"/>
+      <c r="D66" s="124"/>
+      <c r="E66" s="134"/>
       <c r="F66" s="22">
         <v>0.85399999999999998</v>
       </c>
@@ -6619,7 +6619,7 @@
       <c r="D67" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E67" s="125"/>
+      <c r="E67" s="135"/>
       <c r="F67" s="22">
         <v>0.82899999999999996</v>
       </c>
@@ -6651,11 +6651,11 @@
       <c r="B68" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C68" s="126" t="s">
+      <c r="C68" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D68" s="126"/>
-      <c r="E68" s="123" t="s">
+      <c r="D68" s="124"/>
+      <c r="E68" s="133" t="s">
         <v>242</v>
       </c>
       <c r="F68" s="22">
@@ -6695,7 +6695,7 @@
       <c r="D69" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E69" s="124"/>
+      <c r="E69" s="134"/>
       <c r="F69" s="22">
         <v>0.73199999999999998</v>
       </c>
@@ -6727,11 +6727,11 @@
       <c r="B70" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C70" s="126" t="s">
+      <c r="C70" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D70" s="126"/>
-      <c r="E70" s="124"/>
+      <c r="D70" s="124"/>
+      <c r="E70" s="134"/>
       <c r="F70" s="22">
         <v>0.85399999999999998</v>
       </c>
@@ -6769,7 +6769,7 @@
       <c r="D71" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E71" s="124"/>
+      <c r="E71" s="134"/>
       <c r="F71" s="22">
         <v>0.81699999999999995</v>
       </c>
@@ -6801,11 +6801,11 @@
       <c r="B72" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C72" s="126" t="s">
+      <c r="C72" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D72" s="126"/>
-      <c r="E72" s="124"/>
+      <c r="D72" s="124"/>
+      <c r="E72" s="134"/>
       <c r="F72" s="22">
         <v>0.85399999999999998</v>
       </c>
@@ -6843,7 +6843,7 @@
       <c r="D73" s="114" t="s">
         <v>253</v>
       </c>
-      <c r="E73" s="124"/>
+      <c r="E73" s="134"/>
       <c r="F73" s="72" t="s">
         <v>254</v>
       </c>
@@ -6881,7 +6881,7 @@
       <c r="D74" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E74" s="124"/>
+      <c r="E74" s="134"/>
       <c r="F74" s="22">
         <v>0.89</v>
       </c>
@@ -6913,11 +6913,11 @@
       <c r="B75" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C75" s="126" t="s">
+      <c r="C75" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D75" s="126"/>
-      <c r="E75" s="124"/>
+      <c r="D75" s="124"/>
+      <c r="E75" s="134"/>
       <c r="F75" s="22">
         <v>0.878</v>
       </c>
@@ -6955,7 +6955,7 @@
       <c r="D76" s="114" t="s">
         <v>263</v>
       </c>
-      <c r="E76" s="124"/>
+      <c r="E76" s="134"/>
       <c r="F76" s="72" t="s">
         <v>264</v>
       </c>
@@ -6993,7 +6993,7 @@
       <c r="D77" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="E77" s="125"/>
+      <c r="E77" s="135"/>
       <c r="F77" s="22">
         <v>0.90200000000000002</v>
       </c>
@@ -7019,16 +7019,16 @@
       </c>
     </row>
     <row r="78" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="121" t="s">
+      <c r="A78" s="120" t="s">
         <v>271</v>
       </c>
       <c r="B78" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C78" s="126" t="s">
+      <c r="C78" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D78" s="126"/>
+      <c r="D78" s="124"/>
       <c r="E78" s="6" t="s">
         <v>273</v>
       </c>
@@ -7060,14 +7060,14 @@
       </c>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A79" s="121"/>
+      <c r="A79" s="120"/>
       <c r="B79" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C79" s="131" t="s">
+      <c r="C79" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="D79" s="131"/>
+      <c r="D79" s="125"/>
       <c r="E79" s="6" t="s">
         <v>276</v>
       </c>
@@ -7099,14 +7099,14 @@
       </c>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A80" s="121"/>
+      <c r="A80" s="120"/>
       <c r="B80" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C80" s="131" t="s">
+      <c r="C80" s="125" t="s">
         <v>97</v>
       </c>
-      <c r="D80" s="131"/>
+      <c r="D80" s="125"/>
       <c r="E80" s="6" t="s">
         <v>279</v>
       </c>
@@ -7138,16 +7138,16 @@
       </c>
     </row>
     <row r="81" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="121" t="s">
+      <c r="A81" s="120" t="s">
         <v>282</v>
       </c>
       <c r="B81" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C81" s="126" t="s">
+      <c r="C81" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D81" s="126"/>
+      <c r="D81" s="124"/>
       <c r="E81" s="6" t="s">
         <v>283</v>
       </c>
@@ -7179,14 +7179,14 @@
       </c>
     </row>
     <row r="82" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A82" s="121"/>
+      <c r="A82" s="120"/>
       <c r="B82" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="C82" s="126" t="s">
+      <c r="C82" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="D82" s="126"/>
+      <c r="D82" s="124"/>
       <c r="E82" s="6" t="s">
         <v>287</v>
       </c>
@@ -7216,14 +7216,14 @@
       <c r="P82" s="6"/>
     </row>
     <row r="83" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A83" s="121"/>
+      <c r="A83" s="120"/>
       <c r="B83" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C83" s="131" t="s">
+      <c r="C83" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="D83" s="131"/>
+      <c r="D83" s="125"/>
       <c r="E83" s="6" t="s">
         <v>288</v>
       </c>
@@ -7255,14 +7255,14 @@
       </c>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A84" s="121"/>
+      <c r="A84" s="120"/>
       <c r="B84" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="C84" s="131" t="s">
+      <c r="C84" s="125" t="s">
         <v>92</v>
       </c>
-      <c r="D84" s="131"/>
+      <c r="D84" s="125"/>
       <c r="E84" s="6" t="s">
         <v>291</v>
       </c>
@@ -7292,14 +7292,14 @@
       <c r="P84" s="6"/>
     </row>
     <row r="85" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A85" s="121"/>
+      <c r="A85" s="120"/>
       <c r="B85" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C85" s="131" t="s">
+      <c r="C85" s="125" t="s">
         <v>97</v>
       </c>
-      <c r="D85" s="131"/>
+      <c r="D85" s="125"/>
       <c r="E85" s="6" t="s">
         <v>293</v>
       </c>
@@ -7331,16 +7331,16 @@
       </c>
     </row>
     <row r="86" spans="1:18" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="121" t="s">
+      <c r="A86" s="120" t="s">
         <v>296</v>
       </c>
       <c r="B86" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="C86" s="133" t="s">
+      <c r="C86" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="D86" s="133"/>
+      <c r="D86" s="131"/>
       <c r="E86" s="6" t="s">
         <v>298</v>
       </c>
@@ -7370,14 +7370,14 @@
       <c r="P86" s="21"/>
     </row>
     <row r="87" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A87" s="121"/>
+      <c r="A87" s="120"/>
       <c r="B87" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="C87" s="127" t="s">
+      <c r="C87" s="126" t="s">
         <v>92</v>
       </c>
-      <c r="D87" s="127"/>
+      <c r="D87" s="126"/>
       <c r="E87" s="6" t="s">
         <v>300</v>
       </c>
@@ -7407,14 +7407,14 @@
       <c r="P87" s="21"/>
     </row>
     <row r="88" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A88" s="121"/>
+      <c r="A88" s="120"/>
       <c r="B88" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="C88" s="127" t="s">
+      <c r="C88" s="126" t="s">
         <v>92</v>
       </c>
-      <c r="D88" s="127"/>
+      <c r="D88" s="126"/>
       <c r="E88" s="6" t="s">
         <v>303</v>
       </c>
@@ -7444,14 +7444,14 @@
       <c r="P88" s="21"/>
     </row>
     <row r="89" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A89" s="121"/>
+      <c r="A89" s="120"/>
       <c r="B89" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="C89" s="127" t="s">
+      <c r="C89" s="126" t="s">
         <v>97</v>
       </c>
-      <c r="D89" s="127"/>
+      <c r="D89" s="126"/>
       <c r="E89" s="6" t="s">
         <v>305</v>
       </c>
@@ -7481,16 +7481,16 @@
       <c r="P89" s="21"/>
     </row>
     <row r="90" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="121" t="s">
+      <c r="A90" s="120" t="s">
         <v>307</v>
       </c>
       <c r="B90" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="C90" s="131" t="s">
+      <c r="C90" s="125" t="s">
         <v>309</v>
       </c>
-      <c r="D90" s="131"/>
+      <c r="D90" s="125"/>
       <c r="E90" s="5"/>
       <c r="F90" s="30">
         <v>0.86</v>
@@ -7524,7 +7524,7 @@
       <c r="R90" s="2"/>
     </row>
     <row r="91" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A91" s="121"/>
+      <c r="A91" s="120"/>
       <c r="B91" s="21" t="s">
         <v>308</v>
       </c>
@@ -7567,14 +7567,14 @@
       <c r="R91" s="2"/>
     </row>
     <row r="92" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="121"/>
+      <c r="A92" s="120"/>
       <c r="B92" s="21" t="s">
         <v>315</v>
       </c>
-      <c r="C92" s="132" t="s">
+      <c r="C92" s="130" t="s">
         <v>313</v>
       </c>
-      <c r="D92" s="132"/>
+      <c r="D92" s="130"/>
       <c r="E92" s="75"/>
       <c r="F92" s="30">
         <v>0.89</v>
@@ -7608,7 +7608,7 @@
       <c r="R92" s="2"/>
     </row>
     <row r="93" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A93" s="121"/>
+      <c r="A93" s="120"/>
       <c r="B93" s="21" t="s">
         <v>315</v>
       </c>
@@ -7651,8 +7651,8 @@
       <c r="R93" s="2"/>
     </row>
     <row r="94" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A94" s="121"/>
-      <c r="B94" s="128" t="s">
+      <c r="A94" s="120"/>
+      <c r="B94" s="127" t="s">
         <v>315</v>
       </c>
       <c r="C94" s="5" t="s">
@@ -7691,8 +7691,8 @@
       <c r="R94" s="2"/>
     </row>
     <row r="95" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A95" s="121"/>
-      <c r="B95" s="129"/>
+      <c r="A95" s="120"/>
+      <c r="B95" s="128"/>
       <c r="C95" s="5" t="s">
         <v>313</v>
       </c>
@@ -7726,8 +7726,8 @@
       <c r="R95" s="2"/>
     </row>
     <row r="96" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A96" s="121"/>
-      <c r="B96" s="130"/>
+      <c r="A96" s="120"/>
+      <c r="B96" s="129"/>
       <c r="C96" s="5" t="s">
         <v>313</v>
       </c>
@@ -7763,7 +7763,7 @@
       <c r="R96" s="2"/>
     </row>
     <row r="97" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A97" s="121"/>
+      <c r="A97" s="120"/>
       <c r="B97" s="21" t="s">
         <v>315</v>
       </c>
@@ -7803,7 +7803,7 @@
       <c r="R97" s="2"/>
     </row>
     <row r="98" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A98" s="121"/>
+      <c r="A98" s="120"/>
       <c r="B98" s="21" t="s">
         <v>315</v>
       </c>
@@ -7841,7 +7841,7 @@
       <c r="R98" s="2"/>
     </row>
     <row r="99" spans="1:18" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="121" t="s">
+      <c r="A99" s="120" t="s">
         <v>344</v>
       </c>
       <c r="B99" s="21" t="s">
@@ -7883,7 +7883,7 @@
       <c r="R99" s="2"/>
     </row>
     <row r="100" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A100" s="121"/>
+      <c r="A100" s="120"/>
       <c r="B100" s="21" t="s">
         <v>345</v>
       </c>
@@ -7923,7 +7923,7 @@
       <c r="R100" s="2"/>
     </row>
     <row r="101" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A101" s="121"/>
+      <c r="A101" s="120"/>
       <c r="B101" s="21" t="s">
         <v>349</v>
       </c>
@@ -7963,7 +7963,7 @@
       <c r="R101" s="2"/>
     </row>
     <row r="102" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A102" s="121"/>
+      <c r="A102" s="120"/>
       <c r="B102" s="21"/>
       <c r="C102" s="16"/>
       <c r="D102" s="5"/>
@@ -8040,7 +8040,7 @@
         <v>357</v>
       </c>
       <c r="P104" s="78"/>
-      <c r="Q104" s="122" t="s">
+      <c r="Q104" s="132" t="s">
         <v>358</v>
       </c>
     </row>
@@ -8083,7 +8083,7 @@
         <v>357</v>
       </c>
       <c r="P105" s="78"/>
-      <c r="Q105" s="122"/>
+      <c r="Q105" s="132"/>
     </row>
     <row r="106" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A106" s="46" t="s">
@@ -8124,7 +8124,7 @@
         <v>364</v>
       </c>
       <c r="P106" s="78"/>
-      <c r="Q106" s="122" t="s">
+      <c r="Q106" s="132" t="s">
         <v>365</v>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
         <v>364</v>
       </c>
       <c r="P107" s="78"/>
-      <c r="Q107" s="122"/>
+      <c r="Q107" s="132"/>
     </row>
     <row r="108" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A108" s="46" t="s">
@@ -8208,7 +8208,7 @@
         <v>370</v>
       </c>
       <c r="P108" s="78"/>
-      <c r="Q108" s="122" t="s">
+      <c r="Q108" s="132" t="s">
         <v>371</v>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
         <v>370</v>
       </c>
       <c r="P109" s="78"/>
-      <c r="Q109" s="122"/>
+      <c r="Q109" s="132"/>
     </row>
     <row r="110" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A110" s="46" t="s">
@@ -13688,18 +13688,31 @@
   </sheetData>
   <autoFilter ref="A2:P2" xr:uid="{C5C2BC2A-39EF-41BF-AD8A-98A78C1356E2}"/>
   <mergeCells count="53">
-    <mergeCell ref="A99:A102"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="A33:A49"/>
-    <mergeCell ref="A78:A80"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="A90:A98"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="Q106:Q107"/>
+    <mergeCell ref="Q108:Q109"/>
+    <mergeCell ref="E50:E58"/>
+    <mergeCell ref="E68:E77"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="E59:E67"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="Q104:Q105"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
+    <mergeCell ref="C92:D92"/>
+    <mergeCell ref="C90:D90"/>
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="C86:D86"/>
+    <mergeCell ref="C87:D87"/>
+    <mergeCell ref="C88:D88"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="C80:D80"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="C48:D48"/>
@@ -13716,31 +13729,18 @@
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="C62:D62"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="C72:D72"/>
-    <mergeCell ref="C82:D82"/>
-    <mergeCell ref="C83:D83"/>
-    <mergeCell ref="C84:D84"/>
-    <mergeCell ref="C92:D92"/>
-    <mergeCell ref="C90:D90"/>
-    <mergeCell ref="C85:D85"/>
-    <mergeCell ref="C86:D86"/>
-    <mergeCell ref="C87:D87"/>
-    <mergeCell ref="C88:D88"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="C89:D89"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="Q106:Q107"/>
-    <mergeCell ref="Q108:Q109"/>
-    <mergeCell ref="E50:E58"/>
-    <mergeCell ref="E68:E77"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="E59:E67"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="Q104:Q105"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="A99:A102"/>
+    <mergeCell ref="A29:A32"/>
+    <mergeCell ref="A33:A49"/>
+    <mergeCell ref="A78:A80"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="A90:A98"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13768,20 +13768,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="136" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="120"/>
-      <c r="C1" s="120"/>
-      <c r="D1" s="120"/>
-      <c r="E1" s="120"/>
-      <c r="F1" s="120"/>
-      <c r="G1" s="120"/>
-      <c r="H1" s="120"/>
-      <c r="I1" s="120"/>
-      <c r="J1" s="120"/>
-      <c r="K1" s="120"/>
-      <c r="L1" s="120"/>
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="136"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="35" t="s">
@@ -14601,7 +14601,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="121" t="s">
+      <c r="A23" s="120" t="s">
         <v>86</v>
       </c>
       <c r="B23" s="21" t="s">
@@ -14638,7 +14638,7 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="121"/>
+      <c r="A24" s="120"/>
       <c r="B24" s="21" t="s">
         <v>87</v>
       </c>
@@ -14675,7 +14675,7 @@
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="121"/>
+      <c r="A25" s="120"/>
       <c r="B25" s="21" t="s">
         <v>87</v>
       </c>
@@ -14710,7 +14710,7 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="121"/>
+      <c r="A26" s="120"/>
       <c r="B26" s="21" t="s">
         <v>87</v>
       </c>
@@ -14745,7 +14745,7 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="121"/>
+      <c r="A27" s="120"/>
       <c r="B27" s="21" t="s">
         <v>87</v>
       </c>
@@ -14783,7 +14783,7 @@
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" s="121"/>
+      <c r="A28" s="120"/>
       <c r="B28" s="21" t="s">
         <v>87</v>
       </c>
@@ -14818,7 +14818,7 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="121"/>
+      <c r="A29" s="120"/>
       <c r="B29" s="21" t="s">
         <v>87</v>
       </c>
@@ -14853,7 +14853,7 @@
       </c>
     </row>
     <row r="30" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="121" t="s">
+      <c r="A30" s="120" t="s">
         <v>271</v>
       </c>
       <c r="B30" s="21" t="s">
@@ -14890,7 +14890,7 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" s="121"/>
+      <c r="A31" s="120"/>
       <c r="B31" s="21" t="s">
         <v>272</v>
       </c>
@@ -14925,7 +14925,7 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="121"/>
+      <c r="A32" s="120"/>
       <c r="B32" s="21" t="s">
         <v>272</v>
       </c>
@@ -14960,7 +14960,7 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="121"/>
+      <c r="A33" s="120"/>
       <c r="B33" s="21" t="s">
         <v>272</v>
       </c>
@@ -14995,7 +14995,7 @@
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="121"/>
+      <c r="A34" s="120"/>
       <c r="B34" s="21" t="s">
         <v>272</v>
       </c>
@@ -15030,7 +15030,7 @@
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="121"/>
+      <c r="A35" s="120"/>
       <c r="B35" s="21" t="s">
         <v>272</v>
       </c>
@@ -15065,7 +15065,7 @@
       </c>
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="121" t="s">
+      <c r="A36" s="120" t="s">
         <v>296</v>
       </c>
       <c r="B36" s="21" t="s">
@@ -15085,7 +15085,7 @@
       <c r="L36" s="21"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="121"/>
+      <c r="A37" s="120"/>
       <c r="B37" s="21" t="s">
         <v>297</v>
       </c>
@@ -15118,7 +15118,7 @@
       <c r="L37" s="21"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="121"/>
+      <c r="A38" s="120"/>
       <c r="B38" s="21" t="s">
         <v>297</v>
       </c>
@@ -15151,7 +15151,7 @@
       <c r="L38" s="21"/>
     </row>
     <row r="39" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="121" t="s">
+      <c r="A39" s="120" t="s">
         <v>307</v>
       </c>
       <c r="B39" s="21" t="s">
@@ -15192,7 +15192,7 @@
       <c r="N39" s="2"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="121"/>
+      <c r="A40" s="120"/>
       <c r="B40" s="21" t="s">
         <v>308</v>
       </c>
@@ -15233,7 +15233,7 @@
       <c r="N40" s="2"/>
     </row>
     <row r="41" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="121"/>
+      <c r="A41" s="120"/>
       <c r="B41" s="21" t="s">
         <v>315</v>
       </c>
@@ -15271,7 +15271,7 @@
       <c r="N41" s="2"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="121"/>
+      <c r="A42" s="120"/>
       <c r="B42" s="21" t="s">
         <v>315</v>
       </c>
@@ -15308,7 +15308,7 @@
       <c r="N42" s="2"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="121"/>
+      <c r="A43" s="120"/>
       <c r="B43" s="21" t="s">
         <v>315</v>
       </c>
@@ -15360,7 +15360,7 @@
       <c r="N44" s="2"/>
     </row>
     <row r="45" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="121" t="s">
+      <c r="A45" s="120" t="s">
         <v>344</v>
       </c>
       <c r="B45" s="21" t="s">
@@ -15399,7 +15399,7 @@
       <c r="N45" s="2"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="121"/>
+      <c r="A46" s="120"/>
       <c r="B46" s="21" t="s">
         <v>345</v>
       </c>
@@ -15436,7 +15436,7 @@
       <c r="N46" s="2"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="121"/>
+      <c r="A47" s="120"/>
       <c r="B47" s="21" t="s">
         <v>349</v>
       </c>
@@ -18976,6 +18976,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005323BDF9AD652343A74746E7EAA0DAA6" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9f08d66e012038210b9c986140cd53a8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d31a0228-6921-4820-bdaa-a4c82afcfcbc" xmlns:ns3="5ae73a50-db4c-43f8-ae46-ae1a2c7129ce" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e463efb1defe95352308313adaa5d5d" ns2:_="" ns3:_="">
     <xsd:import namespace="d31a0228-6921-4820-bdaa-a4c82afcfcbc"/>
@@ -19210,15 +19219,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAC2F4A9-AFF4-4EEA-BDD9-AF9135ABA11B}">
   <ds:schemaRefs>
@@ -19231,6 +19231,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67511F64-F1D9-4530-A060-7B2D3B766653}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A80E4EC-F71E-492B-91D8-8B4413B53B40}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19247,12 +19255,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67511F64-F1D9-4530-A060-7B2D3B766653}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>